<commit_message>
Penilaian kerja per aspek, fasilitas, dan mode gratis
- Kartu 'Cocok buat kerja?' di halaman kafe: 8 aspek dengan label otomatis dan catatan opsional
- Daftar fasilitas: ada / tidak / belum dicek
- Form admin & sinkron spreadsheet (kolom nilai_*, catatan_*, ada_*); rating keseluruhan otomatis dari rata-rata
- Mode gratis (default aktif): konten terbuka untuk semua, harga/trial/langganan disembunyikan, toggle di Admin > Pengaturan
- Migrasi 0007

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013wknHBqEyU1L5pC8nHKU4Y
</commit_message>
<xml_diff>
--- a/public/template-workfromcafe.xlsx
+++ b/public/template-workfromcafe.xlsx
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -117,6 +117,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -332,6 +333,106 @@
     <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <t>Catatan saja, tidak disinkron.</t>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0" shapeId="0">
+      <text>
+        <t>Kecepatan internet. Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AI1" authorId="0" shapeId="0">
+      <text>
+        <t>Colokan. Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Ketenangan (5 = setenang perpustakaan). Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AK1" authorId="0" shapeId="0">
+      <text>
+        <t>Kenyamanan kursi. Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AL1" authorId="0" shapeId="0">
+      <text>
+        <t>Rasa kopi. Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AM1" authorId="0" shapeId="0">
+      <text>
+        <t>Kebersihan toilet. Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AN1" authorId="0" shapeId="0">
+      <text>
+        <t>Pelayanan. Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AO1" authorId="0" shapeId="0">
+      <text>
+        <t>Harga sepadan. Angka 1–5 (boleh ,5). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AP1" authorId="0" shapeId="0">
+      <text>
+        <t>Internet / Wi-Fi: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AQ1" authorId="0" shapeId="0">
+      <text>
+        <t>Colokan: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AR1" authorId="0" shapeId="0">
+      <text>
+        <t>Parkir: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AS1" authorId="0" shapeId="0">
+      <text>
+        <t>Ruang meeting: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AT1" authorId="0" shapeId="0">
+      <text>
+        <t>Mushola: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AU1" authorId="0" shapeId="0">
+      <text>
+        <t>Makanan berat: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AV1" authorId="0" shapeId="0">
+      <text>
+        <t>Ruangan AC: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AW1" authorId="0" shapeId="0">
+      <text>
+        <t>Area outdoor: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AX1" authorId="0" shapeId="0">
+      <text>
+        <t>Area merokok: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AY1" authorId="0" shapeId="0">
+      <text>
+        <t>Meja berdiri: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="AZ1" authorId="0" shapeId="0">
+      <text>
+        <t>Ramah hewan: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
+      </text>
+    </comment>
+    <comment ref="BA1" authorId="0" shapeId="0">
+      <text>
+        <t>Ada musik: ya / tidak / ? (belum dicek). Kosong = tidak diubah.</t>
       </text>
     </comment>
   </commentList>
@@ -672,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG300"/>
+  <dimension ref="A1:BA300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -708,6 +809,26 @@
     <col width="30" customWidth="1" min="31" max="31"/>
     <col width="16" customWidth="1" min="32" max="32"/>
     <col width="30" customWidth="1" min="33" max="33"/>
+    <col width="15" customWidth="1" min="34" max="34"/>
+    <col width="15" customWidth="1" min="35" max="35"/>
+    <col width="15" customWidth="1" min="36" max="36"/>
+    <col width="15" customWidth="1" min="37" max="37"/>
+    <col width="15" customWidth="1" min="38" max="38"/>
+    <col width="15" customWidth="1" min="39" max="39"/>
+    <col width="15" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="19" customWidth="1" min="45" max="45"/>
+    <col width="13" customWidth="1" min="46" max="46"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="48" max="48"/>
+    <col width="13" customWidth="1" min="49" max="49"/>
+    <col width="18" customWidth="1" min="50" max="50"/>
+    <col width="18" customWidth="1" min="51" max="51"/>
+    <col width="17" customWidth="1" min="52" max="52"/>
+    <col width="12" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -876,6 +997,106 @@
           <t>catatan_internal</t>
         </is>
       </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_internet</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_colokan</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_ketenangan</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_kursi</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_kopi</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_toilet</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_pelayanan</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>nilai_harga</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>ada_wifi</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>ada_colokan</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>ada_parkir</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>ada_ruang_meeting</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>ada_mushola</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>ada_makanan_berat</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>ada_ac</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>ada_outdoor</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>ada_area_merokok</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>ada_meja_berdiri</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>ada_ramah_hewan</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>ada_musik</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -11343,7 +11564,7 @@
       <c r="AG300" s="6" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation sqref="C2:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Referensi!$A$2:$A$30</formula1>
     </dataValidation>
@@ -11358,6 +11579,12 @@
     </dataValidation>
     <dataValidation sqref="AF2:AF300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Belum dikunjungi,Sudah dikunjungi,Tutup permanen"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH2:AH300 AI2:AI300 AJ2:AJ300 AK2:AK300 AL2:AL300 AM2:AM300 AN2:AN300 AO2:AO300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,1.5,2,2.5,3,3.5,4,4.5,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AP2:AP300 AQ2:AQ300 AR2:AR300 AS2:AS300 AT2:AT300 AU2:AU300 AV2:AV300 AW2:AW300 AX2:AX300 AY2:AY300 AZ2:AZ300 BA2:BA300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ya,tidak,?"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15931,7 +16158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -16079,6 +16306,41 @@
     </row>
     <row r="25">
       <c r="A25" s="9" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Penilaian kerja &amp; fasilitas (kolom paling kanan di tab Kafe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>• nilai_internet … nilai_harga: angka 1–5 (boleh 3,5). Keterangan seperti "Cepat" atau "Melimpah" muncul otomatis di aplikasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>• Kalau kolom rating dikosongkan, rating keseluruhan dihitung otomatis dari rata-rata nilai_….</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>• ada_wifi … ada_musik: isi ya, tidak, atau ? (belum dicek).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>• Opsional: tambah kolom catatan_internet, catatan_colokan, dst. untuk menulis keterangan sendiri (maks. 90 huruf), misalnya "50 Mbps, stabil".</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Perluas cakupan ke kota-kota besar Pulau Jawa
- Teks beranda, judul/SEO, manifest PWA, gambar share, peta, komunitas: Pulau Jawa
- Daftar provinsi Jawa + tebak provinsi otomatis dari koordinat (admin kota, sinkron sheet, rekomendasi author)
- Pilihan kota dikelompokkan per provinsi (Jelajah & form author)
- Peta otomatis menyesuaikan ke sebaran kafe
- Migrasi 0010: kota besar se-Jawa (nonaktif sampai ada kafe tayang)
- Template spreadsheet: daftar kota se-Jawa, kota lain tetap boleh

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013wknHBqEyU1L5pC8nHKU4Y
</commit_message>
<xml_diff>
--- a/public/template-workfromcafe.xlsx
+++ b/public/template-workfromcafe.xlsx
@@ -11566,7 +11566,7 @@
   </sheetData>
   <dataValidations count="7">
     <dataValidation sqref="C2:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referensi!$A$2:$A$30</formula1>
+      <formula1>Referensi!$A$2:$A$27</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"10K–30K,20K–40K,30K–50K,40K–60K,60K ke atas"</formula1>
@@ -16353,7 +16353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -16393,7 +16393,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Semarang</t>
+          <t>Jakarta</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
@@ -16420,7 +16420,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Solo</t>
+          <t>Tangerang</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -16447,7 +16447,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Purwokerto</t>
+          <t>Tangerang Selatan</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -16474,7 +16474,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Magelang</t>
+          <t>Serang</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -16501,7 +16501,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Salatiga</t>
+          <t>Bogor</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -16523,7 +16523,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Pekalongan</t>
+          <t>Depok</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -16540,7 +16540,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Tegal</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -16552,31 +16552,152 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
+          <t>Bandung</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Cirebon</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Tasikmalaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Semarang</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Solo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Purwokerto</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Magelang</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Salatiga</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pekalongan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tegal</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Kudus</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Klaten</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Purwodadi</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Yogyakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Surabaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Malang</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sidoarjo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Kediri</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Jember</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Tag baru di kolom suasana/fasilitas dibuat otomatis saat sinkron.</t>
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Kota lain di luar daftar juga boleh; dibuat otomatis saat sinkron (provinsi ditebak dari koordinat).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>